<commit_message>
make ssu64xl a little bit cleaner
</commit_message>
<xml_diff>
--- a/coretp/plans/ssu64xl/SSU64XL_TP.xlsx
+++ b/coretp/plans/ssu64xl/SSU64XL_TP.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B709BE-DB3B-1348-A2C4-38C3589C22AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE8C629-2704-4146-BC64-2C9C84ED7321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="34560" windowHeight="20480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="(NEEDS REWORK) -High Level Plan" sheetId="3" state="hidden" r:id="rId1"/>
@@ -2695,9 +2695,6 @@
     <t>UXL bit check</t>
   </si>
   <si>
-    <t>underflow CSR and do 64 checks with SRLI, verifiying LSB is bit 1 (except after the 64th bit, where it is bit 0)</t>
-  </si>
-  <si>
     <t>Works best if test is ran from U mode. Can only be ran in virtualized/hypervisor mode</t>
   </si>
   <si>
@@ -2755,31 +2752,32 @@
 assert_uxl_h = AssertEqual(src1=uxl_value_h, src2=expected_uxl)</t>
   </si>
   <si>
+    <t>SID_SSU64XL_01</t>
+  </si>
+  <si>
+    <t>SID_SSU64XL_02</t>
+  </si>
+  <si>
+    <t>SID_SSU64XL_03</t>
+  </si>
+  <si>
+    <t>underflow CSR and do word level checks with SRLI, verifiying all bits aret1 (except after the 64th bit, where it is bit 0)</t>
+  </si>
+  <si>
     <t># Load a register with maximum 64-bit value
 test_val = LoadImmediateStep(imm=0xFFFFFFFFFFFFFFFF)
 # Loop 64 times, shifting right and checking LSB
-for i in range(64):
+for i in range(3):
+    bit_shift_amt = i * 16
     # Shift right logical by i positions
-    shift_amt = LoadImmediateStep(imm=i)
+    shift_amt = LoadImmediateStep(imm=bit_shift_amt)
     shifted = Arithmetic(op="srl", src1=test_val, src2=shift_amt)
     # Extract LSB (bit 0)
-    lsb_mask = LoadImmediateStep(imm=1)
+    lsb_mask = LoadImmediateStep(imm=0xFFFF)
     lsb = Arithmetic(op="and", src1=shifted, src2=lsb_mask)
     # Expected value: 1 for bits 0-63, 0 for bit 64+
-    if i &lt; 64:
-        expected_lsb = LoadImmediateStep(imm=1)
-    else:
-        expected_lsb = LoadImmediateStep(imm=0)
+    expected_lsb = LoadImmediateStep(imm=0xFFFF)
     assert_lsb = AssertEqual(src1=lsb, src2=expected_lsb)</t>
-  </si>
-  <si>
-    <t>SID_SSU64XL_01</t>
-  </si>
-  <si>
-    <t>SID_SSU64XL_02</t>
-  </si>
-  <si>
-    <t>SID_SSU64XL_03</t>
   </si>
 </sst>
 </file>
@@ -6115,62 +6113,62 @@
         <v>399</v>
       </c>
       <c r="F2" s="126" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="320" x14ac:dyDescent="0.2">
       <c r="A3" s="127" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B3" s="128" t="s">
         <v>400</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D3" s="28" t="s">
         <v>401</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F3" s="73" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="288" x14ac:dyDescent="0.2">
       <c r="A4" s="127" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B4" s="128" t="s">
         <v>402</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F4" s="73"/>
     </row>
-    <row r="5" spans="1:6" ht="256" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="224" x14ac:dyDescent="0.2">
       <c r="A5" s="127" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B5" s="128" t="s">
         <v>403</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="D5" s="28" t="s">
         <v>401</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="F5" s="73"/>
     </row>
@@ -9847,17 +9845,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e8037ae1-f799-41f0-b119-cbea2f4ab5d4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b3c44bb9-2631-4400-93cf-11acafc6ee3a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100815CC0311B58BB469E58C0B9C6D5A1E3" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="79a74086c6d14e17ca0b97ab053cb4af">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e8037ae1-f799-41f0-b119-cbea2f4ab5d4" xmlns:ns3="b3c44bb9-2631-4400-93cf-11acafc6ee3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c06d79a7380883090ce51ef752d1b9ec" ns2:_="" ns3:_="">
     <xsd:import namespace="e8037ae1-f799-41f0-b119-cbea2f4ab5d4"/>
@@ -10106,6 +10093,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e8037ae1-f799-41f0-b119-cbea2f4ab5d4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b3c44bb9-2631-4400-93cf-11acafc6ee3a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ABFC864-393E-4901-8914-CCD2E06169F8}">
   <ds:schemaRefs>
@@ -10115,17 +10113,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD82851F-30FE-46A1-AAEC-BAC70E7E8825}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e8037ae1-f799-41f0-b119-cbea2f4ab5d4"/>
-    <ds:schemaRef ds:uri="b3c44bb9-2631-4400-93cf-11acafc6ee3a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0B41E4C-9AE0-4937-AB3D-889EDC8FE8D1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10142,4 +10129,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD82851F-30FE-46A1-AAEC-BAC70E7E8825}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e8037ae1-f799-41f0-b119-cbea2f4ab5d4"/>
+    <ds:schemaRef ds:uri="b3c44bb9-2631-4400-93cf-11acafc6ee3a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>